<commit_message>
fix: finish talisman pickups and combat hazard feedback
Unify Bonus body absorption and synchronize authored enemy throws.
Fix route-aware projectiles, helper contacts, ship firing, ramp framing,
and seagull warnings, landing, damage and spinning knockback.

Include runtime assets, focused tests, authoring tools and measured evidence.
</commit_message>
<xml_diff>
--- a/Assets/ShooterSurvival/GameData/Editor/Data.xlsx
+++ b/Assets/ShooterSurvival/GameData/Editor/Data.xlsx
@@ -30976,7 +30976,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="J11" s="24" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="K11" s="24" t="n">
         <x:v>11.9</x:v>
@@ -31033,7 +31033,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="J12" s="24" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="K12" s="24" t="n">
         <x:v>11.9</x:v>
@@ -31075,7 +31075,7 @@
         <x:v>SR18_L_E06_T065_Enemy_YllowMan_Net</x:v>
       </x:c>
       <x:c r="E13" s="23" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F13" s="24" t="str">
         <x:v>공격 반복</x:v>
@@ -31156,15 +31156,15 @@
         <x:v>왼쪽 적보다 체력 15% 증가. 접근 시차를 두고 발동.</x:v>
       </x:c>
       <x:c r="M14" s="29" t="str">
-        <x:v>Normal</x:v>
+        <x:v>Boss</x:v>
       </x:c>
       <x:c r="N14" s="30" t="n">
         <x:f>N13</x:f>
         <x:v>8</x:v>
       </x:c>
       <x:c r="O14" s="30" t="n">
-        <x:f>ROUND(O13*(1+P14),0)</x:f>
-        <x:v>199</x:v>
+        <x:f>ROUND(O13*3,0)</x:f>
+        <x:v>519</x:v>
       </x:c>
       <x:c r="P14" s="31" t="n">
         <x:v>0.15</x:v>
@@ -31306,22 +31306,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F17" s="24" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G17" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H17" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I17" s="24" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J17" s="24" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K17" s="24" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L17" s="21" t="str">
         <x:v>공격력·체력은 밸런스 조정 시트에서 계산.</x:v>
@@ -31361,22 +31361,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F18" s="24" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G18" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H18" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I18" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J18" s="24" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K18" s="24" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L18" s="21" t="str">
         <x:v>왼쪽 적보다 체력 15% 증가. 접근 시차를 두고 발동.</x:v>
@@ -31760,22 +31760,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F25" s="24" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G25" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H25" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I25" s="24" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J25" s="24" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K25" s="24" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L25" s="21" t="str">
         <x:v>공격력·체력은 밸런스 조정 시트에서 계산.</x:v>
@@ -31815,22 +31815,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F26" s="24" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G26" s="24" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H26" s="24" t="n">
-        <x:v>8</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I26" s="24" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J26" s="24" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K26" s="24" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L26" s="21" t="str">
         <x:v>왼쪽 적보다 체력 15% 증가. 접근 시차를 두고 발동.</x:v>
@@ -32340,7 +32340,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="J35" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="K35" t="n">
         <x:v>11.9</x:v>
@@ -32397,7 +32397,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="J36" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="K36" t="n">
         <x:v>11.9</x:v>
@@ -33126,22 +33126,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F49" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G49" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H49" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I49" t="n">
         <x:v>16</x:v>
       </x:c>
       <x:c r="J49" t="n">
-        <x:v>0.8</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K49" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L49" t="str">
         <x:v>공격력·체력은 밸런스 조정 시트에서 계산.</x:v>
@@ -33181,22 +33181,22 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="F50" t="str">
-        <x:v>전방 매복 사격</x:v>
+        <x:v>사격</x:v>
       </x:c>
       <x:c r="G50" t="n">
-        <x:v>3</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="H50" t="n">
-        <x:v>4</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="I50" t="n">
-        <x:v>12</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="J50" t="n">
-        <x:v>1.05</x:v>
+        <x:v>0.62</x:v>
       </x:c>
       <x:c r="K50" t="n">
-        <x:v>11.9</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="L50" t="str">
         <x:v>왼쪽 적보다 체력 15% 증가. 접근 시차를 두고 발동.</x:v>
@@ -33290,7 +33290,7 @@
         <x:v>SR18_L_E25_T293_Enemy_Woman_Right</x:v>
       </x:c>
       <x:c r="E52" t="n">
-        <x:v>1</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="F52" t="str">
         <x:v>공격 반복</x:v>

</xml_diff>

<commit_message>
feat: apply chapter improvements and account progress saving
</commit_message>
<xml_diff>
--- a/Assets/ShooterSurvival/GameData/Editor/Data.xlsx
+++ b/Assets/ShooterSurvival/GameData/Editor/Data.xlsx
@@ -33293,7 +33293,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
-  <dimension ref="B1:Y211"/>
+  <dimension ref="B1:Y235"/>
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
     <col min="2" max="2" width="64" customWidth="1"/>
@@ -37587,6 +37587,366 @@
       </c>
       <c r="F211">
         <v>0</v>
+      </c>
+    </row>
+    <row r="212" spans="2:4">
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>playerSpeed_Jamsil</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D212">
+        <v>7.8</v>
+      </c>
+    </row>
+    <row r="213" spans="2:4">
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>playerSpeed_ShoeTower</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D213">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="214" spans="2:4">
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>progressCoinPerCheckpoint_Jamsil</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D214">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="215" spans="2:4">
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>progressCoinPerCheckpoint_ShoeTower</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D215">
+        <v>420</v>
+      </c>
+    </row>
+    <row r="216" spans="2:4">
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>firstClearJewels_Jamsil</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D216">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="217" spans="2:4">
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>replayClearJewels_Jamsil</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D217">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="218" spans="2:4">
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>firstClearJewels_ShoeTower</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D218">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="219" spans="2:4">
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>replayClearJewels_ShoeTower</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D219">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="220" spans="2:4">
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>coinPickupRadius_Jamsil</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D220">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="221" spans="2:4">
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>coinPickupRadius_ShoeTower</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D221">
+        <v>3.5</v>
+      </c>
+    </row>
+    <row r="222" spans="2:4">
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>c45_cityHealth</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D222">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="223" spans="2:4">
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>c45_cityDamage</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D223">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="224" spans="2:4">
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>c45_towerHealth</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D224">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="225" spans="2:4">
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>c45_towerDamage</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D225">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="226" spans="2:4">
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>c45_archiveHealth</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D226">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="227" spans="2:4">
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>c45_archiveDamage</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D227">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="228" spans="2:4">
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>c45_targetHealth</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D228">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="229" spans="2:4">
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>c45_captainHealth</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D229">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="230" spans="2:4">
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>c45_warningSeconds</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D230">
+        <v>1.6</v>
+      </c>
+    </row>
+    <row r="231" spans="2:4">
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>c45_sweepSeconds</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D231">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="232" spans="2:4">
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>c45_hazardDamageFraction</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D232">
+        <v>0.08</v>
+      </c>
+    </row>
+    <row r="233" spans="2:4">
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>c45_liftSeconds</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D233">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="234" spans="2:4">
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>c45_shopCoins</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D234">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="235" spans="2:4">
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>towerArchiveCoinReward</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>float</t>
+        </is>
+      </c>
+      <c r="D235">
+        <v>840</v>
       </c>
     </row>
   </sheetData>

</xml_diff>